<commit_message>
feat: cor da linha de conexão pela tensão real do conjunto
A planilha atualizada traz a coluna "Tensão de linha (kV)" (69/138/230/500,
curada a partir dos AO-CE do MPO, 49/54 conjuntos). A linha conjunto->SE
passa a ser colorida por essa tensão na paleta das linhas de transmissão,
em vez de herdar a tensão máxima da subestação de destino — que pintava a
maioria das conexões de vermelho (500 kV) porque os conjuntos entram em
69/138 numa SE cuja rede básica é 500 kV. Sem tensão cadastrada, a linha
fica no cinza neutro da paleta.

A mesma planilha corrige o ponto de conexão do Conjunto Eólico Olho D'Água
de "SE João Câmara II" para "SE João Câmara III".

A ficha do conjunto e a ficha da linha de conexão passam a exibir a tensão;
a legenda do mapa estático ganha a faixa de 69 kV.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/localizacao_conjuntos_ons_aneel.xlsx
+++ b/data/localizacao_conjuntos_ons_aneel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanielNascimento\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanielNascimento\Downloads\data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DE2B1A-9D8E-4E67-8B89-05BB7F76F0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F16E0F-1974-4E0F-A5BF-3B48935E7BC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2195" uniqueCount="1100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2196" uniqueCount="1101">
   <si>
     <t>Conjunto</t>
   </si>
@@ -3335,6 +3335,9 @@
   </si>
   <si>
     <t>SE Extremoz II</t>
+  </si>
+  <si>
+    <t>Tensão de linha (kV)</t>
   </si>
 </sst>
 </file>
@@ -3504,7 +3507,11 @@
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -3646,24 +3653,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ConjuntosLocalizacao" displayName="ConjuntosLocalizacao" ref="A1:M55" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
-  <autoFilter ref="A1:M55" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Conjunto" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{397EC2CC-CFF0-4A66-893F-23770892EC28}" name="id_ons" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Localização (lat, long)" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Município(s)" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{A897DC24-CD27-434B-9885-56C31D8DBCC4}" name="Capacidade instalada" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Qtd. usinas" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{B3FADEA3-476B-423B-BFBD-078453DF30B9}" name="Qtde. aerogeradores" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{080150B9-74AC-4F33-BABC-96D996793DAA}" name="Ponto de conexão" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{D2D2B454-5A92-45C2-8B38-C53495069E40}" name="Agente Proprietário" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{F203D6FC-5548-4775-959B-4C686864F8BB}" name="Agente Operador" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{D6E4FA75-D250-446F-9CF1-19409BC718E1}" name="Ajustamento Operativo" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{67022F59-6D90-42D4-B4AB-D8534A1AC761}" name="Logo - Agente Proprietário" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ConjuntosLocalizacao" displayName="ConjuntosLocalizacao" ref="A1:N55" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="A1:N55" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Conjunto" dataDxfId="13"/>
+    <tableColumn id="13" xr3:uid="{397EC2CC-CFF0-4A66-893F-23770892EC28}" name="id_ons" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Localização (lat, long)" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Município(s)" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{A897DC24-CD27-434B-9885-56C31D8DBCC4}" name="Capacidade instalada" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Qtd. usinas" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{B3FADEA3-476B-423B-BFBD-078453DF30B9}" name="Qtde. aerogeradores" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{080150B9-74AC-4F33-BABC-96D996793DAA}" name="Ponto de conexão" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{C4756FAA-0D5E-469A-A36D-4604512D514B}" name="Tensão de linha (kV)" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{D2D2B454-5A92-45C2-8B38-C53495069E40}" name="Agente Proprietário" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{F203D6FC-5548-4775-959B-4C686864F8BB}" name="Agente Operador" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{D6E4FA75-D250-446F-9CF1-19409BC718E1}" name="Ajustamento Operativo" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{67022F59-6D90-42D4-B4AB-D8534A1AC761}" name="Logo - Agente Proprietário" dataDxfId="2">
       <calculatedColumnFormula>_xlfn.IMAGE("https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcS45OHRB4fKbqi8RV9T0jsJtoZsyHl9jIMOeOQSjqJGnHr2kl4RouCvvdKk&amp;s=10")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{FE09ADC7-DC49-41C3-B7EE-215E0205CEB9}" name="Logo - Agente Operador" dataDxfId="0"/>
+    <tableColumn id="12" xr3:uid="{FE09ADC7-DC49-41C3-B7EE-215E0205CEB9}" name="Logo - Agente Operador" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3902,7 +3910,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.26953125" style="1" bestFit="1" customWidth="1"/>
@@ -3913,15 +3921,16 @@
     <col min="6" max="6" width="14.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="48.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="32.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="109.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="87.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.7265625" style="1"/>
+    <col min="9" max="9" width="20.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="48.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="109.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="87.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -3947,22 +3956,25 @@
         <v>918</v>
       </c>
       <c r="I1" s="12" t="s">
+        <v>1100</v>
+      </c>
+      <c r="J1" s="12" t="s">
         <v>912</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="K1" s="12" t="s">
         <v>913</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="L1" s="12" t="s">
         <v>916</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="M1" s="12" t="s">
         <v>1014</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="N1" s="12" t="s">
         <v>1015</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>858</v>
       </c>
@@ -3987,21 +3999,24 @@
       <c r="H2" s="15" t="s">
         <v>979</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="15">
+        <v>230</v>
+      </c>
+      <c r="J2" s="15" t="s">
         <v>915</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="K2" s="15" t="s">
         <v>914</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="L2" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="M2" s="16" t="s">
         <v>1033</v>
       </c>
-      <c r="M2" s="9"/>
-    </row>
-    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N2" s="9"/>
+    </row>
+    <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>859</v>
       </c>
@@ -4026,23 +4041,26 @@
       <c r="H3" s="15" t="s">
         <v>980</v>
       </c>
-      <c r="I3" s="15" t="s">
-        <v>917</v>
+      <c r="I3" s="15">
+        <v>230</v>
       </c>
       <c r="J3" s="15" t="s">
         <v>917</v>
       </c>
       <c r="K3" s="15" t="s">
+        <v>917</v>
+      </c>
+      <c r="L3" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L3" s="16" t="s">
-        <v>1022</v>
       </c>
       <c r="M3" s="16" t="s">
         <v>1022</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N3" s="16" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="14" t="s">
         <v>906</v>
       </c>
@@ -4067,23 +4085,26 @@
       <c r="H4" s="15" t="s">
         <v>980</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="15">
+        <v>230</v>
+      </c>
+      <c r="J4" s="15" t="s">
         <v>921</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="K4" s="15" t="s">
         <v>922</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="L4" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L4" s="16" t="s">
-        <v>1024</v>
       </c>
       <c r="M4" s="16" t="s">
         <v>1024</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4" s="16" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>907</v>
       </c>
@@ -4108,23 +4129,26 @@
       <c r="H5" s="15" t="s">
         <v>980</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="I5" s="15">
+        <v>230</v>
+      </c>
+      <c r="J5" s="15" t="s">
         <v>921</v>
       </c>
-      <c r="J5" s="15" t="s">
+      <c r="K5" s="15" t="s">
         <v>922</v>
       </c>
-      <c r="K5" s="15" t="s">
+      <c r="L5" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L5" s="16" t="s">
-        <v>1024</v>
       </c>
       <c r="M5" s="16" t="s">
         <v>1024</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N5" s="16" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
         <v>860</v>
       </c>
@@ -4149,21 +4173,24 @@
       <c r="H6" s="15" t="s">
         <v>981</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="15">
+        <v>230</v>
+      </c>
+      <c r="J6" s="15" t="s">
         <v>923</v>
       </c>
-      <c r="J6" s="15" t="s">
+      <c r="K6" s="15" t="s">
         <v>924</v>
       </c>
-      <c r="K6" s="15" t="s">
+      <c r="L6" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L6" s="16" t="s">
+      <c r="M6" s="16" t="s">
         <v>1034</v>
       </c>
-      <c r="M6" s="9"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6" s="9"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
         <v>861</v>
       </c>
@@ -4188,23 +4215,26 @@
       <c r="H7" s="15" t="s">
         <v>982</v>
       </c>
-      <c r="I7" s="15" t="s">
-        <v>925</v>
+      <c r="I7" s="15">
+        <v>230</v>
       </c>
       <c r="J7" s="15" t="s">
         <v>925</v>
       </c>
       <c r="K7" s="15" t="s">
+        <v>925</v>
+      </c>
+      <c r="L7" s="15" t="s">
         <v>1012</v>
-      </c>
-      <c r="L7" s="16" t="s">
-        <v>1017</v>
       </c>
       <c r="M7" s="16" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N7" s="16" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
         <v>862</v>
       </c>
@@ -4229,21 +4259,24 @@
       <c r="H8" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I8" s="15" t="s">
-        <v>926</v>
+      <c r="I8" s="15">
+        <v>138</v>
       </c>
       <c r="J8" s="15" t="s">
         <v>926</v>
       </c>
       <c r="K8" s="15" t="s">
+        <v>926</v>
+      </c>
+      <c r="L8" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L8" s="16" t="s">
+      <c r="M8" s="16" t="s">
         <v>1035</v>
       </c>
-      <c r="M8" s="9"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N8" s="9"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
         <v>863</v>
       </c>
@@ -4268,23 +4301,26 @@
       <c r="H9" s="15" t="s">
         <v>972</v>
       </c>
-      <c r="I9" s="15" t="s">
-        <v>927</v>
+      <c r="I9" s="15">
+        <v>230</v>
       </c>
       <c r="J9" s="15" t="s">
         <v>927</v>
       </c>
       <c r="K9" s="15" t="s">
+        <v>927</v>
+      </c>
+      <c r="L9" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L9" s="16" t="s">
-        <v>1019</v>
       </c>
       <c r="M9" s="16" t="s">
         <v>1019</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N9" s="16" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>864</v>
       </c>
@@ -4309,23 +4345,26 @@
       <c r="H10" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I10" s="15" t="s">
-        <v>928</v>
+      <c r="I10" s="15">
+        <v>138</v>
       </c>
       <c r="J10" s="15" t="s">
         <v>928</v>
       </c>
       <c r="K10" s="15" t="s">
+        <v>928</v>
+      </c>
+      <c r="L10" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L10" s="16" t="s">
-        <v>1032</v>
       </c>
       <c r="M10" s="16" t="s">
         <v>1032</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N10" s="16" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>865</v>
       </c>
@@ -4350,23 +4389,26 @@
       <c r="H11" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I11" s="15" t="s">
-        <v>929</v>
+      <c r="I11" s="15">
+        <v>138</v>
       </c>
       <c r="J11" s="15" t="s">
         <v>929</v>
       </c>
       <c r="K11" s="15" t="s">
+        <v>929</v>
+      </c>
+      <c r="L11" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L11" s="16" t="s">
-        <v>1020</v>
       </c>
       <c r="M11" s="16" t="s">
         <v>1020</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N11" s="16" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="13" t="s">
         <v>866</v>
       </c>
@@ -4391,23 +4433,26 @@
       <c r="H12" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I12" s="15" t="s">
-        <v>927</v>
+      <c r="I12" s="15">
+        <v>138</v>
       </c>
       <c r="J12" s="15" t="s">
         <v>927</v>
       </c>
       <c r="K12" s="15" t="s">
+        <v>927</v>
+      </c>
+      <c r="L12" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L12" s="16" t="s">
-        <v>1019</v>
       </c>
       <c r="M12" s="16" t="s">
         <v>1019</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N12" s="16" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="14" t="s">
         <v>902</v>
       </c>
@@ -4432,23 +4477,26 @@
       <c r="H13" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="15">
+        <v>138</v>
+      </c>
+      <c r="J13" s="15" t="s">
         <v>966</v>
       </c>
-      <c r="J13" s="15" t="s">
+      <c r="K13" s="15" t="s">
         <v>922</v>
       </c>
-      <c r="K13" s="15" t="s">
+      <c r="L13" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L13" s="16" t="s">
+      <c r="M13" s="16" t="s">
         <v>1025</v>
       </c>
-      <c r="M13" s="10" t="s">
+      <c r="N13" s="10" t="s">
         <v>1026</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>867</v>
       </c>
@@ -4473,23 +4521,26 @@
       <c r="H14" s="15" t="s">
         <v>985</v>
       </c>
-      <c r="I14" s="15" t="s">
-        <v>925</v>
+      <c r="I14" s="15">
+        <v>500</v>
       </c>
       <c r="J14" s="15" t="s">
         <v>925</v>
       </c>
       <c r="K14" s="15" t="s">
+        <v>925</v>
+      </c>
+      <c r="L14" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L14" s="16" t="s">
-        <v>1017</v>
       </c>
       <c r="M14" s="16" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N14" s="16" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>868</v>
       </c>
@@ -4514,21 +4565,24 @@
       <c r="H15" s="15" t="s">
         <v>979</v>
       </c>
-      <c r="I15" s="15" t="s">
-        <v>930</v>
+      <c r="I15" s="15">
+        <v>69</v>
       </c>
       <c r="J15" s="15" t="s">
         <v>930</v>
       </c>
       <c r="K15" s="15" t="s">
+        <v>930</v>
+      </c>
+      <c r="L15" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L15" s="16" t="s">
+      <c r="M15" s="16" t="s">
         <v>1027</v>
       </c>
-      <c r="M15" s="9"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N15" s="9"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
         <v>869</v>
       </c>
@@ -4553,21 +4607,24 @@
       <c r="H16" s="15" t="s">
         <v>979</v>
       </c>
-      <c r="I16" s="15" t="s">
-        <v>930</v>
+      <c r="I16" s="15">
+        <v>69</v>
       </c>
       <c r="J16" s="15" t="s">
         <v>930</v>
       </c>
       <c r="K16" s="15" t="s">
+        <v>930</v>
+      </c>
+      <c r="L16" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L16" s="16" t="s">
+      <c r="M16" s="16" t="s">
         <v>1027</v>
       </c>
-      <c r="M16" s="9"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N16" s="9"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="13" t="s">
         <v>870</v>
       </c>
@@ -4592,21 +4649,24 @@
       <c r="H17" s="15" t="s">
         <v>979</v>
       </c>
-      <c r="I17" s="15" t="s">
-        <v>930</v>
+      <c r="I17" s="15">
+        <v>69</v>
       </c>
       <c r="J17" s="15" t="s">
         <v>930</v>
       </c>
       <c r="K17" s="15" t="s">
+        <v>930</v>
+      </c>
+      <c r="L17" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L17" s="16" t="s">
+      <c r="M17" s="16" t="s">
         <v>1027</v>
       </c>
-      <c r="M17" s="9"/>
-    </row>
-    <row r="18" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N17" s="9"/>
+    </row>
+    <row r="18" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="13" t="s">
         <v>871</v>
       </c>
@@ -4631,23 +4691,26 @@
       <c r="H18" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I18" s="15" t="s">
-        <v>929</v>
+      <c r="I18" s="15">
+        <v>138</v>
       </c>
       <c r="J18" s="15" t="s">
         <v>929</v>
       </c>
       <c r="K18" s="15" t="s">
+        <v>929</v>
+      </c>
+      <c r="L18" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L18" s="16" t="s">
-        <v>1020</v>
       </c>
       <c r="M18" s="16" t="s">
         <v>1020</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N18" s="16" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="13" t="s">
         <v>872</v>
       </c>
@@ -4672,23 +4735,26 @@
       <c r="H19" s="15" t="s">
         <v>987</v>
       </c>
-      <c r="I19" s="15" t="s">
-        <v>914</v>
+      <c r="I19" s="15">
+        <v>69</v>
       </c>
       <c r="J19" s="15" t="s">
         <v>914</v>
       </c>
       <c r="K19" s="15" t="s">
+        <v>914</v>
+      </c>
+      <c r="L19" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L19" s="16" t="s">
-        <v>1030</v>
       </c>
       <c r="M19" s="16" t="s">
         <v>1030</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N19" s="16" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="13" t="s">
         <v>873</v>
       </c>
@@ -4713,23 +4779,26 @@
       <c r="H20" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I20" s="15" t="s">
-        <v>931</v>
+      <c r="I20" s="15">
+        <v>230</v>
       </c>
       <c r="J20" s="15" t="s">
         <v>931</v>
       </c>
       <c r="K20" s="15" t="s">
+        <v>931</v>
+      </c>
+      <c r="L20" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L20" s="16" t="s">
-        <v>1029</v>
       </c>
       <c r="M20" s="16" t="s">
         <v>1029</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N20" s="16" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="13" t="s">
         <v>874</v>
       </c>
@@ -4754,23 +4823,26 @@
       <c r="H21" s="15" t="s">
         <v>987</v>
       </c>
-      <c r="I21" s="15" t="s">
-        <v>927</v>
+      <c r="I21" s="15">
+        <v>230</v>
       </c>
       <c r="J21" s="15" t="s">
         <v>927</v>
       </c>
       <c r="K21" s="15" t="s">
+        <v>927</v>
+      </c>
+      <c r="L21" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L21" s="16" t="s">
-        <v>1019</v>
       </c>
       <c r="M21" s="16" t="s">
         <v>1019</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N21" s="16" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" s="13" t="s">
         <v>875</v>
       </c>
@@ -4795,23 +4867,26 @@
       <c r="H22" s="15" t="s">
         <v>987</v>
       </c>
-      <c r="I22" s="15" t="s">
-        <v>928</v>
+      <c r="I22" s="15">
+        <v>230</v>
       </c>
       <c r="J22" s="15" t="s">
         <v>928</v>
       </c>
       <c r="K22" s="15" t="s">
+        <v>928</v>
+      </c>
+      <c r="L22" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L22" s="16" t="s">
-        <v>1032</v>
       </c>
       <c r="M22" s="16" t="s">
         <v>1032</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N22" s="16" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" s="13" t="s">
         <v>933</v>
       </c>
@@ -4836,23 +4911,26 @@
       <c r="H23" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I23" s="15" t="s">
-        <v>927</v>
+      <c r="I23" s="15">
+        <v>230</v>
       </c>
       <c r="J23" s="15" t="s">
         <v>927</v>
       </c>
       <c r="K23" s="15" t="s">
+        <v>927</v>
+      </c>
+      <c r="L23" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L23" s="16" t="s">
-        <v>1019</v>
       </c>
       <c r="M23" s="16" t="s">
         <v>1019</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N23" s="16" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
         <v>903</v>
       </c>
@@ -4877,21 +4955,24 @@
       <c r="H24" s="15" t="s">
         <v>989</v>
       </c>
-      <c r="I24" s="15" t="s">
-        <v>935</v>
+      <c r="I24" s="15">
+        <v>500</v>
       </c>
       <c r="J24" s="15" t="s">
         <v>935</v>
       </c>
       <c r="K24" s="15" t="s">
+        <v>935</v>
+      </c>
+      <c r="L24" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L24" s="16" t="s">
+      <c r="M24" s="16" t="s">
         <v>1036</v>
       </c>
-      <c r="M24" s="9"/>
-    </row>
-    <row r="25" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N24" s="9"/>
+    </row>
+    <row r="25" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="13" t="s">
         <v>876</v>
       </c>
@@ -4916,23 +4997,26 @@
       <c r="H25" s="15" t="s">
         <v>986</v>
       </c>
-      <c r="I25" s="15" t="s">
-        <v>936</v>
+      <c r="I25" s="15">
+        <v>500</v>
       </c>
       <c r="J25" s="15" t="s">
         <v>936</v>
       </c>
       <c r="K25" s="15" t="s">
+        <v>936</v>
+      </c>
+      <c r="L25" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L25" s="16" t="s">
-        <v>1021</v>
       </c>
       <c r="M25" s="16" t="s">
         <v>1021</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N25" s="16" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" s="13" t="s">
         <v>877</v>
       </c>
@@ -4957,23 +5041,26 @@
       <c r="H26" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I26" s="15" t="s">
-        <v>929</v>
+      <c r="I26" s="15">
+        <v>138</v>
       </c>
       <c r="J26" s="15" t="s">
         <v>929</v>
       </c>
       <c r="K26" s="15" t="s">
+        <v>929</v>
+      </c>
+      <c r="L26" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L26" s="16" t="s">
-        <v>1020</v>
       </c>
       <c r="M26" s="16" t="s">
         <v>1020</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N26" s="16" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" s="13" t="s">
         <v>878</v>
       </c>
@@ -4998,23 +5085,26 @@
       <c r="H27" s="15" t="s">
         <v>980</v>
       </c>
-      <c r="I27" s="15" t="s">
+      <c r="I27" s="15">
+        <v>138</v>
+      </c>
+      <c r="J27" s="15" t="s">
         <v>937</v>
       </c>
-      <c r="J27" s="15" t="s">
+      <c r="K27" s="15" t="s">
         <v>922</v>
       </c>
-      <c r="K27" s="15" t="s">
+      <c r="L27" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L27" s="16" t="s">
+      <c r="M27" s="16" t="s">
         <v>1037</v>
       </c>
-      <c r="M27" s="10" t="s">
+      <c r="N27" s="10" t="s">
         <v>1038</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
         <v>908</v>
       </c>
@@ -5039,23 +5129,26 @@
       <c r="H28" s="15" t="s">
         <v>980</v>
       </c>
-      <c r="I28" s="15" t="s">
-        <v>925</v>
+      <c r="I28" s="15">
+        <v>230</v>
       </c>
       <c r="J28" s="15" t="s">
         <v>925</v>
       </c>
       <c r="K28" s="15" t="s">
+        <v>925</v>
+      </c>
+      <c r="L28" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L28" s="16" t="s">
-        <v>1017</v>
       </c>
       <c r="M28" s="16" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N28" s="16" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" s="13" t="s">
         <v>879</v>
       </c>
@@ -5080,23 +5173,24 @@
       <c r="H29" s="15" t="s">
         <v>972</v>
       </c>
-      <c r="I29" s="15" t="s">
-        <v>931</v>
-      </c>
+      <c r="I29" s="15"/>
       <c r="J29" s="15" t="s">
         <v>931</v>
       </c>
       <c r="K29" s="15" t="s">
+        <v>931</v>
+      </c>
+      <c r="L29" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L29" s="16" t="s">
-        <v>1029</v>
       </c>
       <c r="M29" s="16" t="s">
         <v>1029</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N29" s="16" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" s="13" t="s">
         <v>880</v>
       </c>
@@ -5121,23 +5215,26 @@
       <c r="H30" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I30" s="15" t="s">
-        <v>936</v>
+      <c r="I30" s="15">
+        <v>230</v>
       </c>
       <c r="J30" s="15" t="s">
         <v>936</v>
       </c>
       <c r="K30" s="15" t="s">
+        <v>936</v>
+      </c>
+      <c r="L30" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L30" s="16" t="s">
-        <v>1021</v>
       </c>
       <c r="M30" s="16" t="s">
         <v>1021</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N30" s="16" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="13" t="s">
         <v>881</v>
       </c>
@@ -5162,23 +5259,26 @@
       <c r="H31" s="15" t="s">
         <v>986</v>
       </c>
-      <c r="I31" s="15" t="s">
-        <v>928</v>
+      <c r="I31" s="15">
+        <v>500</v>
       </c>
       <c r="J31" s="15" t="s">
         <v>928</v>
       </c>
       <c r="K31" s="15" t="s">
+        <v>928</v>
+      </c>
+      <c r="L31" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L31" s="16" t="s">
-        <v>1032</v>
       </c>
       <c r="M31" s="16" t="s">
         <v>1032</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N31" s="16" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" s="13" t="s">
         <v>882</v>
       </c>
@@ -5203,23 +5303,24 @@
       <c r="H32" s="15" t="s">
         <v>972</v>
       </c>
-      <c r="I32" s="15" t="s">
-        <v>929</v>
-      </c>
+      <c r="I32" s="15"/>
       <c r="J32" s="15" t="s">
         <v>929</v>
       </c>
       <c r="K32" s="15" t="s">
+        <v>929</v>
+      </c>
+      <c r="L32" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L32" s="16" t="s">
-        <v>1020</v>
       </c>
       <c r="M32" s="16" t="s">
         <v>1020</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N32" s="16" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>905</v>
       </c>
@@ -5244,23 +5345,26 @@
       <c r="H33" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I33" s="15" t="s">
-        <v>929</v>
+      <c r="I33" s="15">
+        <v>138</v>
       </c>
       <c r="J33" s="15" t="s">
         <v>929</v>
       </c>
       <c r="K33" s="15" t="s">
+        <v>929</v>
+      </c>
+      <c r="L33" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L33" s="16" t="s">
-        <v>1020</v>
       </c>
       <c r="M33" s="16" t="s">
         <v>1020</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N33" s="16" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="14" t="s">
         <v>904</v>
       </c>
@@ -5285,23 +5389,26 @@
       <c r="H34" s="15" t="s">
         <v>982</v>
       </c>
-      <c r="I34" s="15" t="s">
-        <v>914</v>
+      <c r="I34" s="15">
+        <v>230</v>
       </c>
       <c r="J34" s="15" t="s">
         <v>914</v>
       </c>
       <c r="K34" s="15" t="s">
+        <v>914</v>
+      </c>
+      <c r="L34" s="15" t="s">
         <v>1012</v>
-      </c>
-      <c r="L34" s="16" t="s">
-        <v>1030</v>
       </c>
       <c r="M34" s="16" t="s">
         <v>1030</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N34" s="16" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A35" s="13" t="s">
         <v>883</v>
       </c>
@@ -5326,21 +5433,24 @@
       <c r="H35" s="15" t="s">
         <v>987</v>
       </c>
-      <c r="I35" s="15" t="s">
+      <c r="I35" s="15">
+        <v>230</v>
+      </c>
+      <c r="J35" s="15" t="s">
         <v>942</v>
       </c>
-      <c r="J35" s="15" t="s">
+      <c r="K35" s="15" t="s">
         <v>914</v>
       </c>
-      <c r="K35" s="15" t="s">
+      <c r="L35" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L35" s="16" t="s">
+      <c r="M35" s="16" t="s">
         <v>1039</v>
       </c>
-      <c r="M35" s="9"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N35" s="9"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A36" s="13" t="s">
         <v>884</v>
       </c>
@@ -5365,23 +5475,26 @@
       <c r="H36" s="15" t="s">
         <v>973</v>
       </c>
-      <c r="I36" s="15" t="s">
-        <v>943</v>
+      <c r="I36" s="15">
+        <v>500</v>
       </c>
       <c r="J36" s="15" t="s">
         <v>943</v>
       </c>
       <c r="K36" s="15" t="s">
+        <v>943</v>
+      </c>
+      <c r="L36" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L36" s="16" t="s">
-        <v>1028</v>
       </c>
       <c r="M36" s="16" t="s">
         <v>1028</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N36" s="16" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="13" t="s">
         <v>885</v>
       </c>
@@ -5404,25 +5517,26 @@
         <v>47</v>
       </c>
       <c r="H37" s="15" t="s">
-        <v>972</v>
-      </c>
-      <c r="I37" s="15" t="s">
-        <v>927</v>
-      </c>
+        <v>983</v>
+      </c>
+      <c r="I37" s="15"/>
       <c r="J37" s="15" t="s">
         <v>927</v>
       </c>
       <c r="K37" s="15" t="s">
+        <v>927</v>
+      </c>
+      <c r="L37" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L37" s="16" t="s">
-        <v>1019</v>
       </c>
       <c r="M37" s="16" t="s">
         <v>1019</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N37" s="16" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A38" s="14" t="s">
         <v>909</v>
       </c>
@@ -5447,23 +5561,26 @@
       <c r="H38" s="15" t="s">
         <v>980</v>
       </c>
-      <c r="I38" s="15" t="s">
-        <v>925</v>
+      <c r="I38" s="15">
+        <v>230</v>
       </c>
       <c r="J38" s="15" t="s">
         <v>925</v>
       </c>
       <c r="K38" s="15" t="s">
+        <v>925</v>
+      </c>
+      <c r="L38" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L38" s="16" t="s">
-        <v>1017</v>
       </c>
       <c r="M38" s="16" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N38" s="16" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A39" s="14" t="s">
         <v>910</v>
       </c>
@@ -5488,23 +5605,26 @@
       <c r="H39" s="15" t="s">
         <v>980</v>
       </c>
-      <c r="I39" s="15" t="s">
-        <v>925</v>
+      <c r="I39" s="15">
+        <v>230</v>
       </c>
       <c r="J39" s="15" t="s">
         <v>925</v>
       </c>
       <c r="K39" s="15" t="s">
+        <v>925</v>
+      </c>
+      <c r="L39" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L39" s="16" t="s">
-        <v>1017</v>
       </c>
       <c r="M39" s="16" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N39" s="16" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A40" s="13" t="s">
         <v>886</v>
       </c>
@@ -5529,23 +5649,26 @@
       <c r="H40" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I40" s="15" t="s">
-        <v>943</v>
+      <c r="I40" s="15">
+        <v>138</v>
       </c>
       <c r="J40" s="15" t="s">
         <v>943</v>
       </c>
       <c r="K40" s="15" t="s">
+        <v>943</v>
+      </c>
+      <c r="L40" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L40" s="16" t="s">
-        <v>1028</v>
       </c>
       <c r="M40" s="16" t="s">
         <v>1028</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N40" s="16" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="13" t="s">
         <v>887</v>
       </c>
@@ -5570,21 +5693,24 @@
       <c r="H41" s="15" t="s">
         <v>983</v>
       </c>
-      <c r="I41" s="15" t="s">
-        <v>946</v>
+      <c r="I41" s="15">
+        <v>138</v>
       </c>
       <c r="J41" s="15" t="s">
         <v>946</v>
       </c>
       <c r="K41" s="15" t="s">
+        <v>946</v>
+      </c>
+      <c r="L41" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L41" s="16" t="s">
+      <c r="M41" s="16" t="s">
         <v>1042</v>
       </c>
-      <c r="M41" s="9"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N41" s="9"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A42" s="13" t="s">
         <v>888</v>
       </c>
@@ -5609,21 +5735,24 @@
       <c r="H42" s="15" t="s">
         <v>1099</v>
       </c>
-      <c r="I42" s="15" t="s">
+      <c r="I42" s="15">
+        <v>230</v>
+      </c>
+      <c r="J42" s="15" t="s">
         <v>957</v>
       </c>
-      <c r="J42" s="15" t="s">
+      <c r="K42" s="15" t="s">
         <v>922</v>
       </c>
-      <c r="K42" s="15" t="s">
+      <c r="L42" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L42" s="16" t="s">
+      <c r="M42" s="16" t="s">
         <v>1043</v>
       </c>
-      <c r="M42" s="9"/>
-    </row>
-    <row r="43" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="N42" s="9"/>
+    </row>
+    <row r="43" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A43" s="13" t="s">
         <v>889</v>
       </c>
@@ -5648,23 +5777,26 @@
       <c r="H43" s="15" t="s">
         <v>988</v>
       </c>
-      <c r="I43" s="15" t="s">
-        <v>954</v>
+      <c r="I43" s="15">
+        <v>500</v>
       </c>
       <c r="J43" s="15" t="s">
         <v>954</v>
       </c>
       <c r="K43" s="15" t="s">
+        <v>954</v>
+      </c>
+      <c r="L43" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L43" s="16" t="s">
-        <v>1018</v>
       </c>
       <c r="M43" s="16" t="s">
         <v>1018</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N43" s="16" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="13" t="s">
         <v>890</v>
       </c>
@@ -5689,23 +5821,26 @@
       <c r="H44" s="15" t="s">
         <v>988</v>
       </c>
-      <c r="I44" s="15" t="s">
-        <v>954</v>
+      <c r="I44" s="15">
+        <v>500</v>
       </c>
       <c r="J44" s="15" t="s">
         <v>954</v>
       </c>
       <c r="K44" s="15" t="s">
+        <v>954</v>
+      </c>
+      <c r="L44" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L44" s="16" t="s">
-        <v>1018</v>
       </c>
       <c r="M44" s="16" t="s">
         <v>1018</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N44" s="16" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" s="13" t="s">
         <v>891</v>
       </c>
@@ -5730,23 +5865,24 @@
       <c r="H45" s="15" t="s">
         <v>972</v>
       </c>
-      <c r="I45" s="15" t="s">
-        <v>929</v>
-      </c>
+      <c r="I45" s="15"/>
       <c r="J45" s="15" t="s">
         <v>929</v>
       </c>
       <c r="K45" s="15" t="s">
+        <v>929</v>
+      </c>
+      <c r="L45" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L45" s="16" t="s">
-        <v>1020</v>
       </c>
       <c r="M45" s="16" t="s">
         <v>1020</v>
       </c>
-    </row>
-    <row r="46" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N45" s="16" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A46" s="13" t="s">
         <v>892</v>
       </c>
@@ -5771,23 +5907,26 @@
       <c r="H46" s="15" t="s">
         <v>984</v>
       </c>
-      <c r="I46" s="15" t="s">
-        <v>927</v>
+      <c r="I46" s="15">
+        <v>138</v>
       </c>
       <c r="J46" s="15" t="s">
         <v>927</v>
       </c>
       <c r="K46" s="15" t="s">
+        <v>927</v>
+      </c>
+      <c r="L46" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L46" s="16" t="s">
-        <v>1019</v>
       </c>
       <c r="M46" s="16" t="s">
         <v>1019</v>
       </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N46" s="16" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A47" s="13" t="s">
         <v>893</v>
       </c>
@@ -5812,21 +5951,24 @@
       <c r="H47" s="15" t="s">
         <v>986</v>
       </c>
-      <c r="I47" s="15" t="s">
-        <v>961</v>
+      <c r="I47" s="15">
+        <v>500</v>
       </c>
       <c r="J47" s="15" t="s">
         <v>961</v>
       </c>
       <c r="K47" s="15" t="s">
+        <v>961</v>
+      </c>
+      <c r="L47" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L47" s="16" t="s">
+      <c r="M47" s="16" t="s">
         <v>1040</v>
       </c>
-      <c r="M47" s="9"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N47" s="9"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A48" s="13" t="s">
         <v>894</v>
       </c>
@@ -5851,23 +5993,26 @@
       <c r="H48" s="15" t="s">
         <v>972</v>
       </c>
-      <c r="I48" s="15" t="s">
-        <v>964</v>
+      <c r="I48" s="15">
+        <v>230</v>
       </c>
       <c r="J48" s="15" t="s">
         <v>964</v>
       </c>
       <c r="K48" s="15" t="s">
+        <v>964</v>
+      </c>
+      <c r="L48" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L48" s="16" t="s">
-        <v>1023</v>
       </c>
       <c r="M48" s="16" t="s">
         <v>1023</v>
       </c>
-    </row>
-    <row r="49" spans="1:13" ht="58" x14ac:dyDescent="0.35">
+      <c r="N48" s="16" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="58" x14ac:dyDescent="0.35">
       <c r="A49" s="13" t="s">
         <v>895</v>
       </c>
@@ -5892,23 +6037,26 @@
       <c r="H49" s="15" t="s">
         <v>979</v>
       </c>
-      <c r="I49" s="15" t="s">
+      <c r="I49" s="15">
+        <v>69</v>
+      </c>
+      <c r="J49" s="15" t="s">
         <v>966</v>
       </c>
-      <c r="J49" s="15" t="s">
+      <c r="K49" s="15" t="s">
         <v>967</v>
       </c>
-      <c r="K49" s="15" t="s">
+      <c r="L49" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L49" s="16" t="s">
-        <v>1025</v>
       </c>
       <c r="M49" s="16" t="s">
         <v>1025</v>
       </c>
-    </row>
-    <row r="50" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N49" s="16" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="13" t="s">
         <v>896</v>
       </c>
@@ -5933,23 +6081,26 @@
       <c r="H50" s="1" t="s">
         <v>985</v>
       </c>
-      <c r="I50" s="15" t="s">
+      <c r="I50" s="1">
+        <v>500</v>
+      </c>
+      <c r="J50" s="15" t="s">
         <v>968</v>
       </c>
-      <c r="J50" s="15" t="s">
+      <c r="K50" s="15" t="s">
         <v>914</v>
       </c>
-      <c r="K50" s="15" t="s">
+      <c r="L50" s="15" t="s">
         <v>1012</v>
       </c>
-      <c r="L50" s="16" t="s">
+      <c r="M50" s="16" t="s">
         <v>1031</v>
       </c>
-      <c r="M50" s="16" t="s">
+      <c r="N50" s="16" t="s">
         <v>1030</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A51" s="13" t="s">
         <v>897</v>
       </c>
@@ -5974,23 +6125,26 @@
       <c r="H51" s="1" t="s">
         <v>985</v>
       </c>
-      <c r="I51" s="15" t="s">
-        <v>967</v>
+      <c r="I51" s="1">
+        <v>500</v>
       </c>
       <c r="J51" s="15" t="s">
         <v>967</v>
       </c>
       <c r="K51" s="15" t="s">
+        <v>967</v>
+      </c>
+      <c r="L51" s="15" t="s">
         <v>1012</v>
-      </c>
-      <c r="L51" s="16" t="s">
-        <v>1025</v>
       </c>
       <c r="M51" s="16" t="s">
         <v>1025</v>
       </c>
-    </row>
-    <row r="52" spans="1:13" ht="58" x14ac:dyDescent="0.35">
+      <c r="N51" s="16" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" ht="58" x14ac:dyDescent="0.35">
       <c r="A52" s="13" t="s">
         <v>898</v>
       </c>
@@ -6015,23 +6169,26 @@
       <c r="H52" s="15" t="s">
         <v>973</v>
       </c>
-      <c r="I52" s="15" t="s">
-        <v>954</v>
+      <c r="I52" s="15">
+        <v>500</v>
       </c>
       <c r="J52" s="15" t="s">
         <v>954</v>
       </c>
       <c r="K52" s="15" t="s">
+        <v>954</v>
+      </c>
+      <c r="L52" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L52" s="16" t="s">
-        <v>1018</v>
       </c>
       <c r="M52" s="16" t="s">
         <v>1018</v>
       </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N52" s="16" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A53" s="13" t="s">
         <v>899</v>
       </c>
@@ -6056,21 +6213,22 @@
       <c r="H53" s="15" t="s">
         <v>972</v>
       </c>
-      <c r="I53" s="15" t="s">
+      <c r="I53" s="15"/>
+      <c r="J53" s="15" t="s">
         <v>974</v>
       </c>
-      <c r="J53" s="15" t="s">
+      <c r="K53" s="15" t="s">
         <v>924</v>
       </c>
-      <c r="K53" s="15" t="s">
+      <c r="L53" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L53" s="16" t="s">
+      <c r="M53" s="16" t="s">
         <v>1041</v>
       </c>
-      <c r="M53" s="9"/>
-    </row>
-    <row r="54" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="N53" s="9"/>
+    </row>
+    <row r="54" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A54" s="13" t="s">
         <v>900</v>
       </c>
@@ -6095,23 +6253,26 @@
       <c r="H54" s="15" t="s">
         <v>976</v>
       </c>
-      <c r="I54" s="15" t="s">
-        <v>954</v>
+      <c r="I54" s="15">
+        <v>230</v>
       </c>
       <c r="J54" s="15" t="s">
         <v>954</v>
       </c>
       <c r="K54" s="15" t="s">
+        <v>954</v>
+      </c>
+      <c r="L54" s="15" t="s">
         <v>1013</v>
-      </c>
-      <c r="L54" s="16" t="s">
-        <v>1018</v>
       </c>
       <c r="M54" s="16" t="s">
         <v>1018</v>
       </c>
-    </row>
-    <row r="55" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N54" s="16" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A55" s="13" t="s">
         <v>901</v>
       </c>
@@ -6136,116 +6297,119 @@
       <c r="H55" s="15" t="s">
         <v>972</v>
       </c>
-      <c r="I55" s="15" t="s">
-        <v>964</v>
+      <c r="I55" s="15">
+        <v>230</v>
       </c>
       <c r="J55" s="15" t="s">
         <v>964</v>
       </c>
       <c r="K55" s="15" t="s">
+        <v>964</v>
+      </c>
+      <c r="L55" s="15" t="s">
         <v>1013</v>
       </c>
-      <c r="L55" s="16" t="s">
+      <c r="M55" s="16" t="s">
         <v>1023</v>
       </c>
-      <c r="M55" s="16" t="s">
+      <c r="N55" s="16" t="s">
         <v>1023</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="L7" r:id="rId1" xr:uid="{C82A610F-72EF-4F62-8252-3BD5D316A947}"/>
-    <hyperlink ref="M7" r:id="rId2" xr:uid="{32C6F69C-3D2E-437B-9CC1-F86EE2BEA7F9}"/>
-    <hyperlink ref="L14" r:id="rId3" xr:uid="{43E3178A-06BA-4DA8-B0F2-1AC106F26393}"/>
-    <hyperlink ref="M14" r:id="rId4" xr:uid="{13623CF7-F3DB-4E2D-849B-5DB2D6421E55}"/>
-    <hyperlink ref="L28" r:id="rId5" xr:uid="{B8A6FB58-9E1B-4A17-B5F0-6550D9C6425E}"/>
-    <hyperlink ref="M28" r:id="rId6" xr:uid="{FBECD59D-CD9C-4EB1-B6E9-E7C8A2E173CC}"/>
-    <hyperlink ref="L38" r:id="rId7" xr:uid="{ED3BC623-09FD-4A76-B6B8-BBC35BAC93ED}"/>
-    <hyperlink ref="L39" r:id="rId8" xr:uid="{EF3DBF48-8C1B-4FE6-BA70-0B0466C61E35}"/>
-    <hyperlink ref="M38" r:id="rId9" xr:uid="{40100472-AE8B-4B51-AB45-693B64937972}"/>
-    <hyperlink ref="M39" r:id="rId10" xr:uid="{4FDEF55C-FD50-4239-A7C1-DFCC64F96866}"/>
-    <hyperlink ref="L43" r:id="rId11" xr:uid="{AE7DB812-8DD5-4D66-804D-FD22D70378DB}"/>
-    <hyperlink ref="M43:M44" r:id="rId12" display="https://casadosventos.com.br/assets/uploads/opengraph_3d74643ad4.png" xr:uid="{D9799FC0-A995-42BF-91A9-C43FB0FBB85C}"/>
-    <hyperlink ref="M52" r:id="rId13" xr:uid="{1981C0B6-9E00-4419-9C8D-27932E60303F}"/>
-    <hyperlink ref="M54" r:id="rId14" xr:uid="{4CB8BBF0-11DE-425B-BD19-8D7B16EF6D78}"/>
-    <hyperlink ref="L44" r:id="rId15" xr:uid="{59A4B49B-DC93-44BD-AA62-5AD046A91628}"/>
-    <hyperlink ref="L52" r:id="rId16" xr:uid="{56114D33-4F1E-4556-9FD2-67438E3D88F8}"/>
-    <hyperlink ref="L54" r:id="rId17" xr:uid="{1622F2BC-A2A6-4E4E-80EF-F1DCFF67BDC8}"/>
-    <hyperlink ref="L9" r:id="rId18" xr:uid="{28C57C06-2CDE-4428-9833-407E33FEBB35}"/>
-    <hyperlink ref="M9" r:id="rId19" xr:uid="{1974EF23-543A-419D-93EB-E4BCE928536B}"/>
-    <hyperlink ref="M12" r:id="rId20" xr:uid="{219FFC60-448D-4396-B297-7785B505F458}"/>
-    <hyperlink ref="M21" r:id="rId21" xr:uid="{1814BC87-9476-4AB3-B51B-B93679391EBA}"/>
-    <hyperlink ref="M23" r:id="rId22" xr:uid="{7942BEA7-F54F-4D19-BE80-E2F82ECDC0FB}"/>
-    <hyperlink ref="M37" r:id="rId23" xr:uid="{B7A1B03E-D15C-4CB1-B693-FE018280FF07}"/>
-    <hyperlink ref="M46" r:id="rId24" xr:uid="{BF1C32C6-436F-4B80-A36A-DA7B5D90FBB1}"/>
-    <hyperlink ref="L12" r:id="rId25" xr:uid="{5C231ECC-F25B-4B8F-AF06-DB6322D659DE}"/>
-    <hyperlink ref="L21" r:id="rId26" xr:uid="{2C25DF21-DD6E-435F-A0A4-D4CF1FA480CB}"/>
-    <hyperlink ref="L23" r:id="rId27" xr:uid="{9DE70A33-D7D9-4BBA-85ED-2B64306DD069}"/>
-    <hyperlink ref="L37" r:id="rId28" xr:uid="{C5900606-E8AE-4999-B719-D44F756B7FDC}"/>
-    <hyperlink ref="L46" r:id="rId29" xr:uid="{18AF0DA8-3097-4E97-882B-CB262E3CB542}"/>
-    <hyperlink ref="L11" r:id="rId30" xr:uid="{6C5779E4-B8F8-41EE-8ABF-4A2BCD297EB6}"/>
-    <hyperlink ref="M11" r:id="rId31" xr:uid="{FBEDE726-D40B-430D-8C70-E6FF0989425D}"/>
-    <hyperlink ref="M18" r:id="rId32" xr:uid="{302E16D1-02AF-4D42-AD41-60704AFCBF01}"/>
-    <hyperlink ref="M26" r:id="rId33" xr:uid="{07B4BFF0-9FEC-4C5F-97C3-E5322BB56C74}"/>
-    <hyperlink ref="M32:M33" r:id="rId34" display="https://upload.wikimedia.org/wikipedia/commons/thumb/f/fc/Logo_CPFL_Energia.svg/1280px-Logo_CPFL_Energia.svg.png?utm_source=pt.wikipedia.org&amp;utm_campaign=index&amp;utm_content=thumbnail" xr:uid="{6EC6DE46-38CA-4BCC-BD48-F5D5E2D9BD9C}"/>
-    <hyperlink ref="M45" r:id="rId35" xr:uid="{5F059CA9-ADCD-406C-BA11-0530720FFBB1}"/>
-    <hyperlink ref="L18" r:id="rId36" xr:uid="{173D0675-93B0-4CCD-99A1-21755170A078}"/>
-    <hyperlink ref="L26" r:id="rId37" xr:uid="{3F3EC440-A040-46E4-99E0-C65E9163712F}"/>
-    <hyperlink ref="L32:L33" r:id="rId38" display="https://upload.wikimedia.org/wikipedia/commons/thumb/f/fc/Logo_CPFL_Energia.svg/1280px-Logo_CPFL_Energia.svg.png?utm_source=pt.wikipedia.org&amp;utm_campaign=index&amp;utm_content=thumbnail" xr:uid="{B2D624A4-38BD-4806-8252-244ACFCFB05C}"/>
-    <hyperlink ref="L45" r:id="rId39" xr:uid="{2E2470BB-8298-4711-A0A8-2FC54D703CF6}"/>
-    <hyperlink ref="L25" r:id="rId40" xr:uid="{9A79CF94-7798-40B6-AA95-C9FB897DCE04}"/>
-    <hyperlink ref="M25" r:id="rId41" xr:uid="{786005D9-4FA4-4A29-BCEB-3A566920EC79}"/>
-    <hyperlink ref="M30" r:id="rId42" xr:uid="{1E4A4195-3287-4AFA-BA41-14EA227E7CF2}"/>
-    <hyperlink ref="L30" r:id="rId43" xr:uid="{7CAED218-EE8A-4425-81C4-879D6E609AEA}"/>
-    <hyperlink ref="L3" r:id="rId44" xr:uid="{356086EC-19D7-435E-A25B-64AC8C8D8338}"/>
-    <hyperlink ref="M3" r:id="rId45" xr:uid="{8C35F83C-61D2-4D6E-8368-B89F65FF8FD5}"/>
-    <hyperlink ref="L48" r:id="rId46" xr:uid="{83869297-C48B-4260-8969-BFA73E91345D}"/>
-    <hyperlink ref="M48" r:id="rId47" xr:uid="{F4B964E0-69DB-4790-A85C-52831EDE8F15}"/>
-    <hyperlink ref="M55" r:id="rId48" xr:uid="{C8574021-E25F-4560-BF7C-972F54BA15E1}"/>
-    <hyperlink ref="L55" r:id="rId49" xr:uid="{DC0C986D-7BFB-4361-A447-8415A3B45FF8}"/>
-    <hyperlink ref="L4" r:id="rId50" xr:uid="{8C0149D0-10CD-40F0-9CB5-8F0DA4E37AA6}"/>
-    <hyperlink ref="M4:M5" r:id="rId51" display="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcSJ30U9qhgdFTm4Kzb3nGYLQBmLc6KQinM3ldlco11ziNJoIJWfdrAjPHdQ&amp;s=10" xr:uid="{D18B48E6-58FD-4057-B244-5F71C87173BA}"/>
-    <hyperlink ref="L5" r:id="rId52" xr:uid="{3344255B-019A-44B3-BF70-59B4A1F2BC3E}"/>
-    <hyperlink ref="L13" r:id="rId53" xr:uid="{75ABC0B5-75E7-4BCB-B3D2-251B4F3F1B7F}"/>
-    <hyperlink ref="L49" r:id="rId54" xr:uid="{55307EEA-CD5B-4D22-A01D-E66B40D59C09}"/>
-    <hyperlink ref="L51" r:id="rId55" xr:uid="{C8638593-3DFB-4536-9D3E-52BBEC83C6E5}"/>
-    <hyperlink ref="M49" r:id="rId56" xr:uid="{F08F9549-F563-489B-BC4A-73093282C7EB}"/>
-    <hyperlink ref="M51" r:id="rId57" xr:uid="{CF6B0311-2B3B-4739-8AA6-010F2816CD9C}"/>
-    <hyperlink ref="M13" r:id="rId58" xr:uid="{07B9E181-BC56-403B-B0EC-2AFACE7ED5A3}"/>
-    <hyperlink ref="L15" r:id="rId59" xr:uid="{F77A8464-9CFB-4610-B07F-A8826CFB6DDE}"/>
-    <hyperlink ref="L16:L17" r:id="rId60" display="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQc3P-uwyPtyX9HL9YdZrmSpvyWQPkl3DuiaC2WAs47PO3I9pHFo-jGSMCn&amp;s=10" xr:uid="{FBC8391F-5029-4BBB-A4E3-D650765536B2}"/>
-    <hyperlink ref="L36" r:id="rId61" xr:uid="{431454C9-3740-4F78-8A31-5C69ABB8D5B7}"/>
-    <hyperlink ref="M36" r:id="rId62" xr:uid="{3267D3C4-6192-4F64-8D1C-CF877A878816}"/>
-    <hyperlink ref="M40" r:id="rId63" xr:uid="{B3BBD001-9CE8-4160-BD18-E1C59379AF59}"/>
-    <hyperlink ref="L40" r:id="rId64" xr:uid="{837F3BCF-CF43-438C-B56F-7C7E583EE984}"/>
-    <hyperlink ref="L20" r:id="rId65" xr:uid="{46B99848-3FF2-4790-AB6D-D14B63A5D8BF}"/>
-    <hyperlink ref="M20" r:id="rId66" xr:uid="{E80115F7-A16A-4863-87E6-6530C66A9397}"/>
-    <hyperlink ref="M29" r:id="rId67" xr:uid="{DED450F7-D1EB-4D24-8A7B-B717BC312B89}"/>
-    <hyperlink ref="L29" r:id="rId68" xr:uid="{648A4E67-BC8C-4483-824E-BC95E435A195}"/>
-    <hyperlink ref="L34" r:id="rId69" xr:uid="{5CCDEA2A-E168-4544-8EDF-78564619D18E}"/>
-    <hyperlink ref="M34" r:id="rId70" xr:uid="{20C6E6BE-1C3B-4CE9-A16A-5B3BA79B6523}"/>
-    <hyperlink ref="M50" r:id="rId71" xr:uid="{E05BB0BB-4B2A-43F3-9303-60B9019A4252}"/>
-    <hyperlink ref="M19" r:id="rId72" xr:uid="{29932DF6-303B-4460-A2B1-292708D68AA0}"/>
-    <hyperlink ref="L19" r:id="rId73" xr:uid="{7A349A3C-EF7D-4E44-98D7-67466176DC73}"/>
-    <hyperlink ref="L50" r:id="rId74" xr:uid="{2417408C-B6DB-4B7D-9E89-DB442A22D61E}"/>
-    <hyperlink ref="L10" r:id="rId75" xr:uid="{212AFABA-E30E-455E-B4B7-EAEA7A41D0B9}"/>
-    <hyperlink ref="M10" r:id="rId76" xr:uid="{1107F4A0-929B-4798-A347-440AAF3874F8}"/>
-    <hyperlink ref="L22" r:id="rId77" xr:uid="{E32ABF40-3B13-47A4-9B6C-E7F79E8D7C92}"/>
-    <hyperlink ref="M22" r:id="rId78" xr:uid="{84986ACE-32CA-4DFE-BA75-2460533E5482}"/>
-    <hyperlink ref="L31" r:id="rId79" xr:uid="{BF866212-6CFF-4978-9560-DA360E549AC4}"/>
-    <hyperlink ref="M31" r:id="rId80" xr:uid="{DAD42F76-0AC7-4EE8-A9E2-F86DB436B4CC}"/>
-    <hyperlink ref="L2" r:id="rId81" xr:uid="{148F5255-73D8-4042-8E5B-D7EEAEEF590F}"/>
-    <hyperlink ref="L6" r:id="rId82" xr:uid="{7E0BEA1C-3CCD-483A-8B84-706A7E3F6B94}"/>
-    <hyperlink ref="L8" r:id="rId83" xr:uid="{B8BA2D95-57A7-41B8-B393-09CB759B047D}"/>
-    <hyperlink ref="L24" r:id="rId84" xr:uid="{00B8B51A-2B9E-4A9B-9F27-CB0D99FF4971}"/>
-    <hyperlink ref="L27" r:id="rId85" xr:uid="{671DF4A7-801E-4D15-A177-8EF1EB6B9064}"/>
-    <hyperlink ref="M27" r:id="rId86" xr:uid="{1CD4AA6A-3063-42B5-9962-0E03256A1D3D}"/>
-    <hyperlink ref="L35" r:id="rId87" xr:uid="{4C5B3369-334B-4AB1-BAE2-00C45B16F51A}"/>
-    <hyperlink ref="L47" r:id="rId88" xr:uid="{11367303-9A80-4F3E-9600-12A83E45716C}"/>
-    <hyperlink ref="L53" r:id="rId89" xr:uid="{A6DA4C27-4D84-4459-8BE8-776BFB69FCEC}"/>
-    <hyperlink ref="L41" r:id="rId90" xr:uid="{95C4F347-7597-4889-B4F0-B14CD3536AA5}"/>
-    <hyperlink ref="L42" r:id="rId91" xr:uid="{B0A7230D-FA6C-4F51-BDE6-F1043E2474E4}"/>
+    <hyperlink ref="M7" r:id="rId1" xr:uid="{C82A610F-72EF-4F62-8252-3BD5D316A947}"/>
+    <hyperlink ref="N7" r:id="rId2" xr:uid="{32C6F69C-3D2E-437B-9CC1-F86EE2BEA7F9}"/>
+    <hyperlink ref="M14" r:id="rId3" xr:uid="{43E3178A-06BA-4DA8-B0F2-1AC106F26393}"/>
+    <hyperlink ref="N14" r:id="rId4" xr:uid="{13623CF7-F3DB-4E2D-849B-5DB2D6421E55}"/>
+    <hyperlink ref="M28" r:id="rId5" xr:uid="{B8A6FB58-9E1B-4A17-B5F0-6550D9C6425E}"/>
+    <hyperlink ref="N28" r:id="rId6" xr:uid="{FBECD59D-CD9C-4EB1-B6E9-E7C8A2E173CC}"/>
+    <hyperlink ref="M38" r:id="rId7" xr:uid="{ED3BC623-09FD-4A76-B6B8-BBC35BAC93ED}"/>
+    <hyperlink ref="M39" r:id="rId8" xr:uid="{EF3DBF48-8C1B-4FE6-BA70-0B0466C61E35}"/>
+    <hyperlink ref="N38" r:id="rId9" xr:uid="{40100472-AE8B-4B51-AB45-693B64937972}"/>
+    <hyperlink ref="N39" r:id="rId10" xr:uid="{4FDEF55C-FD50-4239-A7C1-DFCC64F96866}"/>
+    <hyperlink ref="M43" r:id="rId11" xr:uid="{AE7DB812-8DD5-4D66-804D-FD22D70378DB}"/>
+    <hyperlink ref="N43:N44" r:id="rId12" display="https://casadosventos.com.br/assets/uploads/opengraph_3d74643ad4.png" xr:uid="{D9799FC0-A995-42BF-91A9-C43FB0FBB85C}"/>
+    <hyperlink ref="N52" r:id="rId13" xr:uid="{1981C0B6-9E00-4419-9C8D-27932E60303F}"/>
+    <hyperlink ref="N54" r:id="rId14" xr:uid="{4CB8BBF0-11DE-425B-BD19-8D7B16EF6D78}"/>
+    <hyperlink ref="M44" r:id="rId15" xr:uid="{59A4B49B-DC93-44BD-AA62-5AD046A91628}"/>
+    <hyperlink ref="M52" r:id="rId16" xr:uid="{56114D33-4F1E-4556-9FD2-67438E3D88F8}"/>
+    <hyperlink ref="M54" r:id="rId17" xr:uid="{1622F2BC-A2A6-4E4E-80EF-F1DCFF67BDC8}"/>
+    <hyperlink ref="M9" r:id="rId18" xr:uid="{28C57C06-2CDE-4428-9833-407E33FEBB35}"/>
+    <hyperlink ref="N9" r:id="rId19" xr:uid="{1974EF23-543A-419D-93EB-E4BCE928536B}"/>
+    <hyperlink ref="N12" r:id="rId20" xr:uid="{219FFC60-448D-4396-B297-7785B505F458}"/>
+    <hyperlink ref="N21" r:id="rId21" xr:uid="{1814BC87-9476-4AB3-B51B-B93679391EBA}"/>
+    <hyperlink ref="N23" r:id="rId22" xr:uid="{7942BEA7-F54F-4D19-BE80-E2F82ECDC0FB}"/>
+    <hyperlink ref="N37" r:id="rId23" xr:uid="{B7A1B03E-D15C-4CB1-B693-FE018280FF07}"/>
+    <hyperlink ref="N46" r:id="rId24" xr:uid="{BF1C32C6-436F-4B80-A36A-DA7B5D90FBB1}"/>
+    <hyperlink ref="M12" r:id="rId25" xr:uid="{5C231ECC-F25B-4B8F-AF06-DB6322D659DE}"/>
+    <hyperlink ref="M21" r:id="rId26" xr:uid="{2C25DF21-DD6E-435F-A0A4-D4CF1FA480CB}"/>
+    <hyperlink ref="M23" r:id="rId27" xr:uid="{9DE70A33-D7D9-4BBA-85ED-2B64306DD069}"/>
+    <hyperlink ref="M37" r:id="rId28" xr:uid="{C5900606-E8AE-4999-B719-D44F756B7FDC}"/>
+    <hyperlink ref="M46" r:id="rId29" xr:uid="{18AF0DA8-3097-4E97-882B-CB262E3CB542}"/>
+    <hyperlink ref="M11" r:id="rId30" xr:uid="{6C5779E4-B8F8-41EE-8ABF-4A2BCD297EB6}"/>
+    <hyperlink ref="N11" r:id="rId31" xr:uid="{FBEDE726-D40B-430D-8C70-E6FF0989425D}"/>
+    <hyperlink ref="N18" r:id="rId32" xr:uid="{302E16D1-02AF-4D42-AD41-60704AFCBF01}"/>
+    <hyperlink ref="N26" r:id="rId33" xr:uid="{07B4BFF0-9FEC-4C5F-97C3-E5322BB56C74}"/>
+    <hyperlink ref="N32:N33" r:id="rId34" display="https://upload.wikimedia.org/wikipedia/commons/thumb/f/fc/Logo_CPFL_Energia.svg/1280px-Logo_CPFL_Energia.svg.png?utm_source=pt.wikipedia.org&amp;utm_campaign=index&amp;utm_content=thumbnail" xr:uid="{6EC6DE46-38CA-4BCC-BD48-F5D5E2D9BD9C}"/>
+    <hyperlink ref="N45" r:id="rId35" xr:uid="{5F059CA9-ADCD-406C-BA11-0530720FFBB1}"/>
+    <hyperlink ref="M18" r:id="rId36" xr:uid="{173D0675-93B0-4CCD-99A1-21755170A078}"/>
+    <hyperlink ref="M26" r:id="rId37" xr:uid="{3F3EC440-A040-46E4-99E0-C65E9163712F}"/>
+    <hyperlink ref="M32:M33" r:id="rId38" display="https://upload.wikimedia.org/wikipedia/commons/thumb/f/fc/Logo_CPFL_Energia.svg/1280px-Logo_CPFL_Energia.svg.png?utm_source=pt.wikipedia.org&amp;utm_campaign=index&amp;utm_content=thumbnail" xr:uid="{B2D624A4-38BD-4806-8252-244ACFCFB05C}"/>
+    <hyperlink ref="M45" r:id="rId39" xr:uid="{2E2470BB-8298-4711-A0A8-2FC54D703CF6}"/>
+    <hyperlink ref="M25" r:id="rId40" xr:uid="{9A79CF94-7798-40B6-AA95-C9FB897DCE04}"/>
+    <hyperlink ref="N25" r:id="rId41" xr:uid="{786005D9-4FA4-4A29-BCEB-3A566920EC79}"/>
+    <hyperlink ref="N30" r:id="rId42" xr:uid="{1E4A4195-3287-4AFA-BA41-14EA227E7CF2}"/>
+    <hyperlink ref="M30" r:id="rId43" xr:uid="{7CAED218-EE8A-4425-81C4-879D6E609AEA}"/>
+    <hyperlink ref="M3" r:id="rId44" xr:uid="{356086EC-19D7-435E-A25B-64AC8C8D8338}"/>
+    <hyperlink ref="N3" r:id="rId45" xr:uid="{8C35F83C-61D2-4D6E-8368-B89F65FF8FD5}"/>
+    <hyperlink ref="M48" r:id="rId46" xr:uid="{83869297-C48B-4260-8969-BFA73E91345D}"/>
+    <hyperlink ref="N48" r:id="rId47" xr:uid="{F4B964E0-69DB-4790-A85C-52831EDE8F15}"/>
+    <hyperlink ref="N55" r:id="rId48" xr:uid="{C8574021-E25F-4560-BF7C-972F54BA15E1}"/>
+    <hyperlink ref="M55" r:id="rId49" xr:uid="{DC0C986D-7BFB-4361-A447-8415A3B45FF8}"/>
+    <hyperlink ref="M4" r:id="rId50" xr:uid="{8C0149D0-10CD-40F0-9CB5-8F0DA4E37AA6}"/>
+    <hyperlink ref="N4:N5" r:id="rId51" display="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcSJ30U9qhgdFTm4Kzb3nGYLQBmLc6KQinM3ldlco11ziNJoIJWfdrAjPHdQ&amp;s=10" xr:uid="{D18B48E6-58FD-4057-B244-5F71C87173BA}"/>
+    <hyperlink ref="M5" r:id="rId52" xr:uid="{3344255B-019A-44B3-BF70-59B4A1F2BC3E}"/>
+    <hyperlink ref="M13" r:id="rId53" xr:uid="{75ABC0B5-75E7-4BCB-B3D2-251B4F3F1B7F}"/>
+    <hyperlink ref="M49" r:id="rId54" xr:uid="{55307EEA-CD5B-4D22-A01D-E66B40D59C09}"/>
+    <hyperlink ref="M51" r:id="rId55" xr:uid="{C8638593-3DFB-4536-9D3E-52BBEC83C6E5}"/>
+    <hyperlink ref="N49" r:id="rId56" xr:uid="{F08F9549-F563-489B-BC4A-73093282C7EB}"/>
+    <hyperlink ref="N51" r:id="rId57" xr:uid="{CF6B0311-2B3B-4739-8AA6-010F2816CD9C}"/>
+    <hyperlink ref="N13" r:id="rId58" xr:uid="{07B9E181-BC56-403B-B0EC-2AFACE7ED5A3}"/>
+    <hyperlink ref="M15" r:id="rId59" xr:uid="{F77A8464-9CFB-4610-B07F-A8826CFB6DDE}"/>
+    <hyperlink ref="M16:M17" r:id="rId60" display="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQc3P-uwyPtyX9HL9YdZrmSpvyWQPkl3DuiaC2WAs47PO3I9pHFo-jGSMCn&amp;s=10" xr:uid="{FBC8391F-5029-4BBB-A4E3-D650765536B2}"/>
+    <hyperlink ref="M36" r:id="rId61" xr:uid="{431454C9-3740-4F78-8A31-5C69ABB8D5B7}"/>
+    <hyperlink ref="N36" r:id="rId62" xr:uid="{3267D3C4-6192-4F64-8D1C-CF877A878816}"/>
+    <hyperlink ref="N40" r:id="rId63" xr:uid="{B3BBD001-9CE8-4160-BD18-E1C59379AF59}"/>
+    <hyperlink ref="M40" r:id="rId64" xr:uid="{837F3BCF-CF43-438C-B56F-7C7E583EE984}"/>
+    <hyperlink ref="M20" r:id="rId65" xr:uid="{46B99848-3FF2-4790-AB6D-D14B63A5D8BF}"/>
+    <hyperlink ref="N20" r:id="rId66" xr:uid="{E80115F7-A16A-4863-87E6-6530C66A9397}"/>
+    <hyperlink ref="N29" r:id="rId67" xr:uid="{DED450F7-D1EB-4D24-8A7B-B717BC312B89}"/>
+    <hyperlink ref="M29" r:id="rId68" xr:uid="{648A4E67-BC8C-4483-824E-BC95E435A195}"/>
+    <hyperlink ref="M34" r:id="rId69" xr:uid="{5CCDEA2A-E168-4544-8EDF-78564619D18E}"/>
+    <hyperlink ref="N34" r:id="rId70" xr:uid="{20C6E6BE-1C3B-4CE9-A16A-5B3BA79B6523}"/>
+    <hyperlink ref="N50" r:id="rId71" xr:uid="{E05BB0BB-4B2A-43F3-9303-60B9019A4252}"/>
+    <hyperlink ref="N19" r:id="rId72" xr:uid="{29932DF6-303B-4460-A2B1-292708D68AA0}"/>
+    <hyperlink ref="M19" r:id="rId73" xr:uid="{7A349A3C-EF7D-4E44-98D7-67466176DC73}"/>
+    <hyperlink ref="M50" r:id="rId74" xr:uid="{2417408C-B6DB-4B7D-9E89-DB442A22D61E}"/>
+    <hyperlink ref="M10" r:id="rId75" xr:uid="{212AFABA-E30E-455E-B4B7-EAEA7A41D0B9}"/>
+    <hyperlink ref="N10" r:id="rId76" xr:uid="{1107F4A0-929B-4798-A347-440AAF3874F8}"/>
+    <hyperlink ref="M22" r:id="rId77" xr:uid="{E32ABF40-3B13-47A4-9B6C-E7F79E8D7C92}"/>
+    <hyperlink ref="N22" r:id="rId78" xr:uid="{84986ACE-32CA-4DFE-BA75-2460533E5482}"/>
+    <hyperlink ref="M31" r:id="rId79" xr:uid="{BF866212-6CFF-4978-9560-DA360E549AC4}"/>
+    <hyperlink ref="N31" r:id="rId80" xr:uid="{DAD42F76-0AC7-4EE8-A9E2-F86DB436B4CC}"/>
+    <hyperlink ref="M2" r:id="rId81" xr:uid="{148F5255-73D8-4042-8E5B-D7EEAEEF590F}"/>
+    <hyperlink ref="M6" r:id="rId82" xr:uid="{7E0BEA1C-3CCD-483A-8B84-706A7E3F6B94}"/>
+    <hyperlink ref="M8" r:id="rId83" xr:uid="{B8BA2D95-57A7-41B8-B393-09CB759B047D}"/>
+    <hyperlink ref="M24" r:id="rId84" xr:uid="{00B8B51A-2B9E-4A9B-9F27-CB0D99FF4971}"/>
+    <hyperlink ref="M27" r:id="rId85" xr:uid="{671DF4A7-801E-4D15-A177-8EF1EB6B9064}"/>
+    <hyperlink ref="N27" r:id="rId86" xr:uid="{1CD4AA6A-3063-42B5-9962-0E03256A1D3D}"/>
+    <hyperlink ref="M35" r:id="rId87" xr:uid="{4C5B3369-334B-4AB1-BAE2-00C45B16F51A}"/>
+    <hyperlink ref="M47" r:id="rId88" xr:uid="{11367303-9A80-4F3E-9600-12A83E45716C}"/>
+    <hyperlink ref="M53" r:id="rId89" xr:uid="{A6DA4C27-4D84-4459-8BE8-776BFB69FCEC}"/>
+    <hyperlink ref="M41" r:id="rId90" xr:uid="{95C4F347-7597-4889-B4F0-B14CD3536AA5}"/>
+    <hyperlink ref="M42" r:id="rId91" xr:uid="{B0A7230D-FA6C-4F51-BDE6-F1043E2474E4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>